<commit_message>
Add service type to company onboarding
Create/Edit Company now asks for Service Type (AMC, Non-AMC, Regular).
AMC shows an AMC type picker (C AMC / NC AMC) and required start/end
dates; other types hide them. The company list shows the type, and the
AMC Excel template and export gain service_type and amc_type columns.
</commit_message>
<xml_diff>
--- a/evergreen-latest/app/src/main/assets/evergreen_amc_template.xlsx
+++ b/evergreen-latest/app/src/main/assets/evergreen_amc_template.xlsx
@@ -12,123 +12,138 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
-  <si>
-    <t>company_name</t>
-  </si>
-  <si>
-    <t>branch_name</t>
-  </si>
-  <si>
-    <t>company_email</t>
-  </si>
-  <si>
-    <t>company_location</t>
-  </si>
-  <si>
-    <t>start_date</t>
-  </si>
-  <si>
-    <t>end_date</t>
-  </si>
-  <si>
-    <t>admin_name</t>
-  </si>
-  <si>
-    <t>admin_phone</t>
-  </si>
-  <si>
-    <t>admin_email</t>
-  </si>
-  <si>
-    <t>admin_password</t>
-  </si>
-  <si>
-    <t>admin_location</t>
-  </si>
-  <si>
-    <t>Apollo Hospitals</t>
-  </si>
-  <si>
-    <t>Jubilee Hills</t>
-  </si>
-  <si>
-    <t>apollo.jubilee@example.com</t>
-  </si>
-  <si>
-    <t>Hyderabad</t>
-  </si>
-  <si>
-    <t>2026-04-01</t>
-  </si>
-  <si>
-    <t>2027-03-31</t>
-  </si>
-  <si>
-    <t>Ravi Kumar</t>
-  </si>
-  <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>ravi.apollo@example.com</t>
-  </si>
-  <si>
-    <t>Apollo@123</t>
-  </si>
-  <si>
-    <t>KIMS Hospitals</t>
-  </si>
-  <si>
-    <t>Secunderabad</t>
-  </si>
-  <si>
-    <t>kims.sec@example.com</t>
-  </si>
-  <si>
-    <t>2026-01-15</t>
-  </si>
-  <si>
-    <t>2026-12-31</t>
-  </si>
-  <si>
-    <t>Sneha Reddy</t>
-  </si>
-  <si>
-    <t>9123456780</t>
-  </si>
-  <si>
-    <t>sneha.kims@example.com</t>
-  </si>
-  <si>
-    <t>Kims@123</t>
-  </si>
-  <si>
-    <t>How to use this sheet</t>
-  </si>
-  <si>
-    <t>Use the AMCs sheet. Keep the first row headers exactly as they are.</t>
-  </si>
-  <si>
-    <t>Each row creates one AMC/company and its client admin.</t>
-  </si>
-  <si>
-    <t>Required: company_name, branch_name, admin_name, admin_phone, admin_email, admin_password.</t>
-  </si>
-  <si>
-    <t>admin_phone must be a 10-digit Indian mobile number.</t>
-  </si>
-  <si>
-    <t>Optional: company_email, company_location, start_date, end_date (YYYY-MM-DD), admin_location.</t>
-  </si>
-  <si>
-    <t>If dates are empty, start_date becomes today and end_date becomes one year later.</t>
-  </si>
-  <si>
-    <t>Do not reuse a company+branch pair or an existing admin phone/email.</t>
-  </si>
-  <si>
-    <t>Delete the sample rows before uploading real data, or change phones/emails so they are unique.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+  <si>
+    <t xml:space="preserve">company_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">branch_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">company_email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">company_location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">service_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amc_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">start_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">end_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_location</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apollo Hospitals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jubilee Hills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apollo.jubilee@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hyderabad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C AMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027-03-31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ravi Kumar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9876543210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ravi.apollo@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apollo@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KIMS Hospitals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secunderabad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kims.sec@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-AMC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sneha Reddy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9123456780</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sneha.kims@example.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kims@123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to use this sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use the AMCs sheet. Keep the first row headers exactly as they are.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each row creates one company and its client admin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required: company_name, branch_name, admin_name, admin_phone, admin_email, admin_password.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin_phone must be a 10-digit Indian mobile number.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">service_type: AMC, Non-AMC or Regular. Empty means AMC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amc_type: C AMC or NC AMC. Required when service_type is AMC; leave empty for Non-AMC and Regular.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">start_date, end_date (YYYY-MM-DD) are used only for AMC. If empty, start_date becomes today and end_date one year later.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional: company_email, company_location, admin_location.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do not reuse a company+branch pair or an existing admin phone/email.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete the sample rows before uploading real data, or change phones/emails so they are unique.</t>
   </si>
 </sst>
 </file>
@@ -531,23 +546,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -581,138 +599,155 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M3" t="s">
         <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1">
       <c r="A1" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>